<commit_message>
Redraw and number submission figures; audit Results against accepted data
Organize nine main figures in Results order, nine supplementary figures and
one supplementary scoring-workflow scheme. Split Vina discrimination from
method differences, add cohort and membership-sensitivity views, correct
the direct-Vina versus OOF labeling, and show matched ranking populations.
Provide embedded-font PDF, editable SVG and 600 dpi PNG, figure source CSVs,
captions, renumbering and a review PDF.

Add Table S9D for CAP5 chemistry sensitivity and synchronize its workbook,
data package and citation index. Record 205 passing Results numerical checks,
558 passing table checks, 97 protected-source checks and graphics QA.
Preserve accepted populations, labels, scores, folds, formal statistics and
original figures. No docking, RMSD, bootstrap, AUROC, ranking or model fitting
is rerun. The author will update the full Results text using the citation map.
</commit_message>
<xml_diff>
--- a/Dual_Target_Docking/submission/02_SI_Tables/Supplementary_Tables.xlsx
+++ b/Dual_Target_Docking/submission/02_SI_Tables/Supplementary_Tables.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1" sheetId="1" r:id="Raa73dc6a07df407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S2" sheetId="2" r:id="Re4347bae1078451c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S3" sheetId="3" r:id="R9d8eb5eaa31a48d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S4" sheetId="4" r:id="R870a4c71760d4bed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S5" sheetId="5" r:id="Rbea62063707c4e5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S6" sheetId="6" r:id="R169302a5d767496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S7" sheetId="7" r:id="R091321badbb24876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S8" sheetId="8" r:id="R47947a5f97354550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S9" sheetId="9" r:id="R1784f9d57f9849a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S10" sheetId="10" r:id="R87420c0495e44891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1" sheetId="1" r:id="R15e8fb758e0e46d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S2" sheetId="2" r:id="R9778dffd93af4820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S3" sheetId="3" r:id="Rcaeefdf73c744cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S4" sheetId="4" r:id="R5084d16497d9475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S5" sheetId="5" r:id="R566d87202688495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S6" sheetId="6" r:id="R405e831e9f604b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S7" sheetId="7" r:id="R7d2738b26ff64572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S8" sheetId="8" r:id="R852727f517ad40b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S9" sheetId="9" r:id="Rd87d2355a3b748ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S10" sheetId="10" r:id="R19b04fd880fb417e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12972,28 +12972,534 @@
         <x:v>0.7366666667</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="21" customHeight="1">
-      <x:c r="A37" s="14" t="str">
+    <x:row r="37">
+      <x:c r="A37" s="2" t="str">
+        <x:v>D. Chemistry-model sensitivity to CAP5</x:v>
+      </x:c>
+      <x:c r="B37" s="2"/>
+      <x:c r="C37" s="2"/>
+      <x:c r="D37" s="2"/>
+      <x:c r="E37" s="2"/>
+      <x:c r="F37" s="2"/>
+      <x:c r="G37" s="2"/>
+      <x:c r="H37" s="2"/>
+      <x:c r="I37" s="2"/>
+    </x:row>
+    <x:row r="38" ht="56" customHeight="1">
+      <x:c r="A38" s="8" t="str">
+        <x:v>Target pair</x:v>
+      </x:c>
+      <x:c r="B38" s="8" t="str">
+        <x:v>Direction</x:v>
+      </x:c>
+      <x:c r="C38" s="8" t="str">
+        <x:v>Original OOF n</x:v>
+      </x:c>
+      <x:c r="D38" s="8" t="str">
+        <x:v>CAP5 OOF n</x:v>
+      </x:c>
+      <x:c r="E38" s="8" t="str">
+        <x:v>Original ECFP4 AUROC</x:v>
+      </x:c>
+      <x:c r="F38" s="8" t="str">
+        <x:v>CAP5 ECFP4 AUROC</x:v>
+      </x:c>
+      <x:c r="G38" s="8" t="str">
+        <x:v>ECFP4 AUROC change</x:v>
+      </x:c>
+      <x:c r="H38" s="8" t="str">
+        <x:v>Original Vina increment</x:v>
+      </x:c>
+      <x:c r="I38" s="8" t="str">
+        <x:v>CAP5 Vina increment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="10" t="str">
+        <x:v>EGFR/HER2</x:v>
+      </x:c>
+      <x:c r="B39" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E39" s="16" t="n">
+        <x:v>0.8001930501930502</x:v>
+      </x:c>
+      <x:c r="F39" s="16" t="n">
+        <x:v>0.8001930501930502</x:v>
+      </x:c>
+      <x:c r="G39" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H39" s="16" t="n">
+        <x:v>-0.016409266409266432</x:v>
+      </x:c>
+      <x:c r="I39" s="16" t="n">
+        <x:v>-0.016409266409266432</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="10" t="str">
+        <x:v>EGFR/HER2</x:v>
+      </x:c>
+      <x:c r="B40" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E40" s="16" t="n">
+        <x:v>0.8790322580645161</x:v>
+      </x:c>
+      <x:c r="F40" s="16" t="n">
+        <x:v>0.8790322580645161</x:v>
+      </x:c>
+      <x:c r="G40" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H40" s="16" t="n">
+        <x:v>-0.0023041474654378336</x:v>
+      </x:c>
+      <x:c r="I40" s="16" t="n">
+        <x:v>-0.0023041474654378336</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="10" t="str">
+        <x:v>JAK1/JAK2</x:v>
+      </x:c>
+      <x:c r="B41" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E41" s="16" t="n">
+        <x:v>0.91845703125</x:v>
+      </x:c>
+      <x:c r="F41" s="16" t="n">
+        <x:v>0.9078663793103449</x:v>
+      </x:c>
+      <x:c r="G41" s="16" t="n">
+        <x:v>-0.010590651939655138</x:v>
+      </x:c>
+      <x:c r="H41" s="16" t="n">
+        <x:v>0.00146484375</x:v>
+      </x:c>
+      <x:c r="I41" s="16" t="n">
+        <x:v>0.004849137931034475</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="10" t="str">
+        <x:v>JAK1/JAK2</x:v>
+      </x:c>
+      <x:c r="B42" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E42" s="16" t="n">
+        <x:v>0.9677734375</x:v>
+      </x:c>
+      <x:c r="F42" s="16" t="n">
+        <x:v>0.9677734375</x:v>
+      </x:c>
+      <x:c r="G42" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H42" s="16" t="n">
+        <x:v>0.0029296875</x:v>
+      </x:c>
+      <x:c r="I42" s="16" t="n">
+        <x:v>0.0029296875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="10" t="str">
+        <x:v>JAK1/TYK2</x:v>
+      </x:c>
+      <x:c r="B43" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D43" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E43" s="16" t="n">
+        <x:v>0.8487903225806451</x:v>
+      </x:c>
+      <x:c r="F43" s="16" t="n">
+        <x:v>0.8487903225806451</x:v>
+      </x:c>
+      <x:c r="G43" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H43" s="16" t="n">
+        <x:v>-0.005040322580645129</x:v>
+      </x:c>
+      <x:c r="I43" s="16" t="n">
+        <x:v>-0.005040322580645129</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="24" customHeight="1">
+      <x:c r="A44" s="10" t="str">
+        <x:v>JAK1/TYK2</x:v>
+      </x:c>
+      <x:c r="B44" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D44" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E44" s="16" t="n">
+        <x:v>0.9042338709677419</x:v>
+      </x:c>
+      <x:c r="F44" s="16" t="n">
+        <x:v>0.9042338709677419</x:v>
+      </x:c>
+      <x:c r="G44" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H44" s="16" t="n">
+        <x:v>-0.0010080645161290036</x:v>
+      </x:c>
+      <x:c r="I44" s="16" t="n">
+        <x:v>-0.0010080645161290036</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="10" t="str">
+        <x:v>PIK3CA/mTOR</x:v>
+      </x:c>
+      <x:c r="B45" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D45" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E45" s="16" t="n">
+        <x:v>0.8212890625</x:v>
+      </x:c>
+      <x:c r="F45" s="16" t="n">
+        <x:v>0.8212890625</x:v>
+      </x:c>
+      <x:c r="G45" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H45" s="16" t="n">
+        <x:v>0.021484375</x:v>
+      </x:c>
+      <x:c r="I45" s="16" t="n">
+        <x:v>0.021484375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="24" customHeight="1">
+      <x:c r="A46" s="10" t="str">
+        <x:v>PIK3CA/mTOR</x:v>
+      </x:c>
+      <x:c r="B46" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D46" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E46" s="16" t="n">
+        <x:v>0.728515625</x:v>
+      </x:c>
+      <x:c r="F46" s="16" t="n">
+        <x:v>0.728515625</x:v>
+      </x:c>
+      <x:c r="G46" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H46" s="16" t="n">
+        <x:v>-0.0029296875</x:v>
+      </x:c>
+      <x:c r="I46" s="16" t="n">
+        <x:v>-0.0029296875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="24" customHeight="1">
+      <x:c r="A47" s="10" t="str">
+        <x:v>AChE/BChE</x:v>
+      </x:c>
+      <x:c r="B47" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D47" s="12" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E47" s="16" t="n">
+        <x:v>0.8992592592592593</x:v>
+      </x:c>
+      <x:c r="F47" s="16" t="n">
+        <x:v>0.8992592592592593</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H47" s="16" t="n">
+        <x:v>-0.004444444444444473</x:v>
+      </x:c>
+      <x:c r="I47" s="16" t="n">
+        <x:v>-0.004444444444444473</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="24" customHeight="1">
+      <x:c r="A48" s="10" t="str">
+        <x:v>AChE/BChE</x:v>
+      </x:c>
+      <x:c r="B48" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D48" s="12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E48" s="16" t="n">
+        <x:v>0.8201058201058201</x:v>
+      </x:c>
+      <x:c r="F48" s="16" t="n">
+        <x:v>0.8201058201058201</x:v>
+      </x:c>
+      <x:c r="G48" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H48" s="16" t="n">
+        <x:v>-0.005291005291005346</x:v>
+      </x:c>
+      <x:c r="I48" s="16" t="n">
+        <x:v>-0.005291005291005346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="24" customHeight="1">
+      <x:c r="A49" s="10" t="str">
+        <x:v>F2/F10</x:v>
+      </x:c>
+      <x:c r="B49" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E49" s="16" t="n">
+        <x:v>0.9405241935483871</x:v>
+      </x:c>
+      <x:c r="F49" s="16" t="n">
+        <x:v>0.9405241935483871</x:v>
+      </x:c>
+      <x:c r="G49" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H49" s="16" t="n">
+        <x:v>-0.007056451612903247</x:v>
+      </x:c>
+      <x:c r="I49" s="16" t="n">
+        <x:v>-0.007056451612903247</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="24" customHeight="1">
+      <x:c r="A50" s="10" t="str">
+        <x:v>F2/F10</x:v>
+      </x:c>
+      <x:c r="B50" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D50" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E50" s="16" t="n">
+        <x:v>0.6633064516129032</x:v>
+      </x:c>
+      <x:c r="F50" s="16" t="n">
+        <x:v>0.6633064516129032</x:v>
+      </x:c>
+      <x:c r="G50" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H50" s="16" t="n">
+        <x:v>0.03629032258064513</x:v>
+      </x:c>
+      <x:c r="I50" s="16" t="n">
+        <x:v>0.03629032258064513</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="24" customHeight="1">
+      <x:c r="A51" s="10" t="str">
+        <x:v>PPARG/PPARA</x:v>
+      </x:c>
+      <x:c r="B51" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D51" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E51" s="16" t="n">
+        <x:v>0.8205645161290323</x:v>
+      </x:c>
+      <x:c r="F51" s="16" t="n">
+        <x:v>0.8205645161290323</x:v>
+      </x:c>
+      <x:c r="G51" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H51" s="16" t="n">
+        <x:v>-0.014112903225806495</x:v>
+      </x:c>
+      <x:c r="I51" s="16" t="n">
+        <x:v>-0.014112903225806495</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="24" customHeight="1">
+      <x:c r="A52" s="10" t="str">
+        <x:v>PPARG/PPARA</x:v>
+      </x:c>
+      <x:c r="B52" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C52" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D52" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E52" s="16" t="n">
+        <x:v>0.6669921875</x:v>
+      </x:c>
+      <x:c r="F52" s="16" t="n">
+        <x:v>0.6669921875</x:v>
+      </x:c>
+      <x:c r="G52" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H52" s="16" t="n">
+        <x:v>-0.005859375</x:v>
+      </x:c>
+      <x:c r="I52" s="16" t="n">
+        <x:v>-0.005859375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="24" customHeight="1">
+      <x:c r="A53" s="10" t="str">
+        <x:v>PPARA/PPARD</x:v>
+      </x:c>
+      <x:c r="B53" s="10" t="str">
+        <x:v>D_vs_A</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E53" s="16" t="n">
+        <x:v>0.931640625</x:v>
+      </x:c>
+      <x:c r="F53" s="16" t="n">
+        <x:v>0.9344758064516129</x:v>
+      </x:c>
+      <x:c r="G53" s="16" t="n">
+        <x:v>0.002835181451612878</x:v>
+      </x:c>
+      <x:c r="H53" s="16" t="n">
+        <x:v>-0.0029296875</x:v>
+      </x:c>
+      <x:c r="I53" s="16" t="n">
+        <x:v>-0.003024193548387122</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="24" customHeight="1">
+      <x:c r="A54" s="10" t="str">
+        <x:v>PPARA/PPARD</x:v>
+      </x:c>
+      <x:c r="B54" s="10" t="str">
+        <x:v>D_vs_B</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E54" s="16" t="n">
+        <x:v>0.8740234375</x:v>
+      </x:c>
+      <x:c r="F54" s="16" t="n">
+        <x:v>0.86875</x:v>
+      </x:c>
+      <x:c r="G54" s="16" t="n">
+        <x:v>-0.005273437499999978</x:v>
+      </x:c>
+      <x:c r="H54" s="16" t="n">
+        <x:v>0.0048828125</x:v>
+      </x:c>
+      <x:c r="I54" s="16" t="n">
+        <x:v>0.004166666666666652</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="21" customHeight="1">
+      <x:c r="A57" s="14" t="str">
         <x:v>CAP5 is post hoc supporting sensitivity: at most five ligands per nonempty Murcko scaffold within pair and activity class; acyclic ligands are</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="21" customHeight="1">
-      <x:c r="A38" s="14" t="str">
+    <x:row r="58" ht="21" customHeight="1">
+      <x:c r="A58" s="14" t="str">
         <x:v>exempt. Six ligands are excluded without replacement. Complete CAP5 method comparisons, chemical models, controls and ranking outputs are retained</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="21" customHeight="1">
-      <x:c r="A39" s="14" t="str">
+    <x:row r="59" ht="21" customHeight="1">
+      <x:c r="A59" s="14" t="str">
         <x:v>in Supplementary_Data.zip. The PPARA/PPARD S5 dual-versus-A-only CI changes from [0.4921875, 0.767578125] to [0.5030241935, 0.7772177419]; this</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="21" customHeight="1">
-      <x:c r="A40" s="14" t="str">
+    <x:row r="60" ht="21" customHeight="1">
+      <x:c r="A60" s="14" t="str">
         <x:v>boundary change is retained, without a general significance claim. The strict Q110 subset has 56 members (25 dual, 12 A-only, 14 B-only, 5</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="21" customHeight="1">
-      <x:c r="A41" s="14" t="str">
+    <x:row r="61" ht="21" customHeight="1">
+      <x:c r="A61" s="14" t="str">
         <x:v>neither). Main and subset populations differ; no new paired CI for their difference is calculated.</x:v>
       </x:c>
     </x:row>

</xml_diff>